<commit_message>
2000/01–2020/21: okresní soutěže z clbs (jen názvy) + oprava CLUBS zápisu
Dokončení okresní úplnosti po současnost (+~1500 klubů). Klíčová oprava nástroje:
list CLUBS má mezi érami RŮZNÉ pořadí sloupců (stará hlavička clean/raw/sheet/
entry_note/level/district/prev vs moderní raw/clean/entry_note/prev/sheet/level),
proto se teď zapisuje podle NÁZVŮ sloupců, ne pozičně – jinak v moderních
souborech příznak 'N' zatékal do prev_club_id. prev 27148, 0 rozbitých.

https://claude.ai/code/session_01BhRGgVD2Sevo7xfvYw5ngZ
</commit_message>
<xml_diff>
--- a/data/S2007_08_FINAL.xlsx
+++ b/data/S2007_08_FINAL.xlsx
@@ -6394,7 +6394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W36"/>
+  <dimension ref="A1:W61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8532,6 +8532,1085 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Krajská liga</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0074</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SB Světlá nad Sázavou</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Krajská liga</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0074</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0196</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00231</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>SKLH Žďár nad Sázavou</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Krajská liga</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0074</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0197</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00232</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>6</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>HC Chotěboř</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Krajská liga</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0074</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0198</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00233</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SK Žamberk</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0199</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00234</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Sokol Tisová</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0200</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00235</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Jiskra Králíky</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0201</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00236</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Sokol Řetová</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0202</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00237</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>HC Dlouhoňovice</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0203</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00238</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>6</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TJ Voděrady</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0204</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00239</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>7</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Sokol Verměřovice</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0205</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00240</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>HC Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0206</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00241</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>9</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Sokol Semanín</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0207</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00242</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Spartak Pelhřimov B</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0208</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00243</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Takže Čejov</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0209</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00244</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>HC Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0210</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00245</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>HC Pelhřimov</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0211</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00246</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>5</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Jiskra Humpolec B</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0212</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00247</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>6</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>HC Buřenice</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0213</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00248</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>7</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>HC Počátky</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0214</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00249</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>8</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>SK Telč B</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0215</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00250</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>9</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>SK Horní Cerekev</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0216</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00251</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>10</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Slavoj Žirovnice</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0217</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00252</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>11</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TJ Růžená</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0218</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00253</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8543,7 +9622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W32"/>
+  <dimension ref="A1:W70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10280,6 +11359,1684 @@
       <c r="V32" t="inlineStr">
         <is>
           <t>SER_S2007_08_0033</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>HC Blansko D</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0219</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00254</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Černá Hora</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0220</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00255</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Rájec – Jestřebí</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0221</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00256</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>4</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Sokol Lysice</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0222</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00257</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>5</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Adamov</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0223</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00258</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Březina</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0224</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00259</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>7</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Letovice</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0225</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00260</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>8</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Kunštát</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0226</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00261</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>9</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Sokol Sloup</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0227</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00262</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Sokol Pokojovice</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0228</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00263</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Sokol Okříšky</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0229</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00264</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Sokol Stařeč</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0230</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00265</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Náměšť nad Oslavou „B“</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0231</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00266</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>5</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Jiskra Vladislav</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0232</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00267</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>6</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TJ Mohelno</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0233</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00268</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>WhiteStar Vizovice</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0234</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00269</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>KASMEN Uherský Brod</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0235</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00270</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Metropol Podkopná Lhota</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0236</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00271</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>HC Napajedla</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0237</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00272</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>5</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>BUM Otrokovice</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0238</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00273</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>6</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Baťovka Zlín</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0239</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00274</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>7</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Rudí kohouti Zlín</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0240</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00275</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>8</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>KAS Asterix Napajedla</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0241</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00276</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Veverská Bitýška</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0242</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00277</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>SK Mostiště</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0243</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00278</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TJ Řečice</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0244</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00279</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>HC Slavkovice</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0245</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00280</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>5</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Spartak Velká Bíteš B</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0246</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00281</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>6</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Náměšť nad Oslavou</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0247</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00282</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>7</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>HC Sokol Křižanov</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0248</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00283</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>8</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>HC Vatín</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0249</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00284</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Šerkovice</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0250</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00285</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Polná</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0251</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00286</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>3</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Měřín</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0252</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00287</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>finále</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0253</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00288</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>SD-CHO 6:6,4:6</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0254</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00289</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>finále: Dvůr-Týniště 7:2</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Blansko</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0255</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>TR_S2007_08_00290</t>
         </is>
       </c>
     </row>
@@ -11298,7 +14055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N88"/>
+  <dimension ref="A1:N91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15287,6 +18044,97 @@
       <c r="A88" t="inlineStr">
         <is>
           <t>II.liga: Západ/Střed/Východ + 8F/QF/SF/finále.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0074</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Pardubický – Krajská liga</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>league</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0075</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Pardubický – Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>league</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0076</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Jihomoravský – Blansko</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>league</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>REG_JHM</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>NODE_S2007_08_0069</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy).</t>
         </is>
       </c>
     </row>
@@ -18922,7 +21770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J184"/>
+  <dimension ref="A1:J244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="10" max="10"/>
@@ -26638,6 +29486,1926 @@
       <c r="J184" t="inlineStr">
         <is>
           <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0196</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>SB Světlá nad Sázavou</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>SB Světlá nad Sázavou</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0197</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>SKLH Žďár nad Sázavou</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>SKLH Žďár nad Sázavou</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0198</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>HC Chotěboř</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>HC Chotěboř</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0199</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>SK Žamberk</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>SK Žamberk</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0200</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Sokol Tisová</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Sokol Tisová</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0201</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Jiskra Králíky</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Jiskra Králíky</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0202</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Sokol Řetová</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Sokol Řetová</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0203</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>HC Dlouhoňovice</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>HC Dlouhoňovice</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0204</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>TJ Voděrady</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>TJ Voděrady</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0205</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Sokol Verměřovice</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Sokol Verměřovice</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0206</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>HC Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>HC Ústí nad Orlicí</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0207</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Sokol Semanín</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Sokol Semanín</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0208</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Spartak Pelhřimov B</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Spartak Pelhřimov B</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0209</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Takže Čejov</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Takže Čejov</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0210</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>HC Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>HC Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0211</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>HC Pelhřimov</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>HC Pelhřimov</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0212</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Jiskra Humpolec B</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Jiskra Humpolec B</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0213</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>HC Buřenice</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>HC Buřenice</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0214</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>HC Počátky</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>HC Počátky</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0215</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>SK Telč B</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>SK Telč B</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0216</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>SK Horní Cerekev</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>SK Horní Cerekev</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0217</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Slavoj Žirovnice</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Slavoj Žirovnice</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0218</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>TJ Růžená</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>TJ Růžená</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>30PARD</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0219</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>HC Blansko D</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>HC Blansko D</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0220</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Černá Hora</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Černá Hora</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0221</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Rájec – Jestřebí</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Rájec – Jestřebí</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0222</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Sokol Lysice</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Sokol Lysice</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0223</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Adamov</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Adamov</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0224</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Březina</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Březina</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0225</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Letovice</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Letovice</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0226</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Kunštát</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Kunštát</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0227</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Sokol Sloup</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Sokol Sloup</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0228</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Sokol Pokojovice</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Sokol Pokojovice</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0229</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Sokol Okříšky</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Sokol Okříšky</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0230</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Sokol Stařeč</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Sokol Stařeč</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0231</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Náměšť nad Oslavou „B“</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Náměšť nad Oslavou „B“</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0232</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Jiskra Vladislav</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Jiskra Vladislav</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0233</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>TJ Mohelno</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>TJ Mohelno</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0234</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>WhiteStar Vizovice</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>WhiteStar Vizovice</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0235</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>KASMEN Uherský Brod</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>KASMEN Uherský Brod</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0236</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Metropol Podkopná Lhota</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Metropol Podkopná Lhota</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0237</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>HC Napajedla</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>HC Napajedla</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0238</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>BUM Otrokovice</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>BUM Otrokovice</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0239</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Baťovka Zlín</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Baťovka Zlín</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0240</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Rudí kohouti Zlín</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Rudí kohouti Zlín</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0241</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>KAS Asterix Napajedla</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>KAS Asterix Napajedla</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0242</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Veverská Bitýška</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Veverská Bitýška</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0243</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>SK Mostiště</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>SK Mostiště</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0244</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>TJ Řečice</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>TJ Řečice</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0245</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>HC Slavkovice</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>HC Slavkovice</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0246</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Spartak Velká Bíteš B</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Spartak Velká Bíteš B</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0247</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Náměšť nad Oslavou</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Náměšť nad Oslavou</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0248</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>HC Sokol Křižanov</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>HC Sokol Křižanov</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0249</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>HC Vatín</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>HC Vatín</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0250</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Šerkovice</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Šerkovice</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0251</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Polná</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Polná</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0252</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Měřín</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Měřín</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0253</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>finále</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>finále</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0254</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>SD-CHO 6:6,4:6</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>SD-CHO 6:6,4:6</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>CLUB_S2007_08_0255</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>finále: Dvůr-Týniště 7:2</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>finále: Dvůr-Týniště 7:2</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>30JHMR</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Okresní soutěž – základ úplnosti z clbs (jen názvy, bez statistik).</t>
         </is>
       </c>
     </row>

</xml_diff>